<commit_message>
chore: Excel 朴素描述版已上传 datadrive.world (PDF 不入库)
</commit_message>
<xml_diff>
--- a/reports/state_space_features.xlsx
+++ b/reports/state_space_features.xlsx
@@ -537,7 +537,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>探测本机 metaworld 数据集根目录与规模</t>
+          <t>数据系统模块负责探测本机 metaworld 数据集, 先确认数据集根目录是否存在且可访问, 再统计其中数据的规模, 以便在训练与评估开始前确认数据资源已经就绪。</t>
         </is>
       </c>
       <c r="H2" t="n">
@@ -586,7 +586,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>metaworld 环境与任务 (peg-insert-side-v3) 加载</t>
+          <t>数据源模块加载 metaworld 仿真环境, 同时载入该环境配套的圆柱销侧向插入任务的第三版, 为整条感知、估计与控制链路准备好统一的仿真运行场景。</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -635,7 +635,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>39D 状态流维数与动作 4D 契约</t>
+          <t>该数据源输出 39 维的状态流，并依据动作空间 4 维的契约对观测维度进行对齐，保证状态流与动作两者的维数约定一致、顺序对应。</t>
         </is>
       </c>
       <c r="H4" t="n">
@@ -684,7 +684,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>数据源 → 数据世界逐帧发布 (画布/3D/总线同源)</t>
+          <t>数据源模块把采集到的每一帧数据逐帧发布到数据世界中去,画布显示、三维空间渲染和总线传输所读到的都是同一份数据,保证三处内容同源一致。</t>
         </is>
       </c>
       <c r="H5" t="n">
@@ -733,7 +733,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>与训练/评估数据链路一致 (LeRobotDataset 兼容)</t>
+          <t>工程数据接入功能保证本模块读取的数据与训练阶段和评估阶段所用的数据链路保持一致，并且数据格式与 LeRobotDataset 数据集格式相兼容。</t>
         </is>
       </c>
       <c r="H6" t="n">
@@ -782,7 +782,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>39D 视觉 + 触觉 4D → 43D (fuse_sensors)</t>
+          <t>传感器融合模块把视觉系统给出的 39 维图像平面观测与触觉系统给出的 4 维触觉观测拼接融合, 合成一个 43 维的统一观测向量, 供统一状态编码环节使用。</t>
         </is>
       </c>
       <c r="H7" t="n">
@@ -831,7 +831,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>当前帧+历史帧 (cur/prev) 时空结构</t>
+          <t>传感器融合模块把当前时刻的观测帧与上一时刻的历史观测帧拼接起来, 构成同时包含时间先后与空间对应关系的上下文结构, 再整体交给状态估计环节使用。</t>
         </is>
       </c>
       <c r="H8" t="n">
@@ -880,7 +880,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>力传感器合成 + 触觉 4D 并入统一向量</t>
+          <t>本模块把力传感器测得的力觉数据与 4 维触觉信号合成在一起，并把合成结果统一并入同一个观测向量，供下游模块取用。</t>
         </is>
       </c>
       <c r="H9" t="n">
@@ -929,7 +929,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>感知来源标记 (编码器/视觉/触觉) 可追溯</t>
+          <t>传感器融合模块为每一条观测数据都打上感知来源的标记,明确指出这条数据来自编码器、视觉还是触觉,让任何一条观测都能追溯到它的来源。</t>
         </is>
       </c>
       <c r="H10" t="n">
@@ -978,7 +978,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>融合计算耗时在播放节奏内 (&lt;30ms)</t>
+          <t>传感器融合功能会把一次融合计算的耗时控制在画面播放节奏允许的时限以内，确保单次融合耗时小于三十毫秒。</t>
         </is>
       </c>
       <c r="H11" t="n">
@@ -1027,7 +1027,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>多源观测编码为单一 43D 向量 (状态空间观测方程)</t>
+          <t>状态编码器按照状态空间的观测方程, 把视觉、触觉等多源传感器送来的观测统一编码为单一的 43 维状态向量, 使机器人各下游模块都基于同一份状态表示开展工作。</t>
         </is>
       </c>
       <c r="H12" t="n">
@@ -1076,7 +1076,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>几何/工件段位 (hand/peg/hole/target)</t>
+          <t>状态估计器把视觉系统识别出的机械手、圆柱销、插孔与目标物这四类对象, 分别按几何属性与工件属性进行分段, 再把各段量测数值映射进统一状态向量的对应位置, 得到完整的场景状态。</t>
         </is>
       </c>
       <c r="H13" t="n">
@@ -1125,7 +1125,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>夹紧度/接触标志嵌入状态向量</t>
+          <t>该模块把夹紧度数值与接触标志这两类信息嵌入 43 维统一状态向量之中，使下游各模块能直接从状态向量里读到这两项触觉信息。</t>
         </is>
       </c>
       <c r="H14" t="n">
@@ -1174,7 +1174,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>模型行/场景结构条件可叠加 (不破坏基础观测)</t>
+          <t>任务模型行条件与场景结构条件都可以叠加到统一的43维状态向量上,而且这种叠加操作不会破坏原本的基础观测数据,保证基础信息始终完整。</t>
         </is>
       </c>
       <c r="H15" t="n">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>每个字段可追溯到编码器/视觉/触觉/真值</t>
+          <t>统一状态向量中的每一个字段都可以追溯到它自己的数据源头，数据源头可能是编码器输出、视觉信息、触觉信息或者真值数据。</t>
         </is>
       </c>
       <c r="H16" t="n">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>蒸馏 MLP 比例引导 (547K 前向学解析教师 Kp·Δ, 训练域内近似; 解析律降级为域外守卫 D_GUARD=0.25)</t>
+          <t>前馈加速器用约 54.7 万参数的动作决策网络做前向推理, 逼近解析教师的比例控制增益乘误差引导律, 在训练域内输出近似引导动作以加快响应; 若状态越出训练域, 解析控制律降级为域外守卫, 把 D_GUARD 标志置为 0.25。</t>
         </is>
       </c>
       <c r="H17" t="n">
@@ -1321,7 +1321,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>接近目标时闭合控制 (近距判据 d_xy&lt;0.03)</t>
+          <t>前馈加速器以机械臂末端与目标之间的平面距离 d_xy 小于 0.03 作为近距离判据, 一旦满足该判据就启动闭合控制, 让末端在接近目标时迅速收敛到期望位置。</t>
         </is>
       </c>
       <c r="H18" t="n">
@@ -1370,7 +1370,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>前馈输出 ±0.6 限幅 (反归一化后 clip; 旧解析律 ±0.5 随主路径退役)</t>
+          <t>前馈加速器的输出在完成反归一化之后会被截断，把幅值限制在正负 0.6 以内；旧的解析控制律按正负 0.5 限幅，现已随主路径一起退役，不再生效。</t>
         </is>
       </c>
       <c r="H19" t="n">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>obs→u_ff 直接映射无递归 (快慢分离之快)</t>
+          <t>前馈加速器把观测数据直接映射为前馈动作量并输出,整个映射过程不做任何递归迭代计算,这正是快慢两条路径分离方案中的快路径,动作响应非常直接迅速。</t>
         </is>
       </c>
       <c r="H20" t="n">
@@ -1468,7 +1468,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>前馈输出有物理含义 (目标方向/大小)</t>
+          <t>前馈加速器输出的动作带有明确的物理含义，例如目标运动方向和目标运动大小，因此使用者能够理解每一个输出的作用。</t>
         </is>
       </c>
       <c r="H21" t="n">
@@ -1517,7 +1517,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>递归潜状态 + 卡尔曼 predict (世界模型)</t>
+          <t>自适应状态估计器以递归方式维护潜状态, 并按世界模型执行卡尔曼滤波的预测步骤, 提前推算下一时刻潜状态的均值与协方差, 为随后到来的观测校正提供先验依据。</t>
         </is>
       </c>
       <c r="H22" t="n">
@@ -1566,7 +1566,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>update 门控: 信预测 vs 信观测 (K 可标定)</t>
+          <t>自适应状态估计器在每次更新时先做门控判断, 根据预测与观测的一致程度决定更相信先验预测还是更相信新到的观测, 并利用可标定的卡尔曼增益 K 调节两者的融合比例。</t>
         </is>
       </c>
       <c r="H23" t="n">
@@ -1615,7 +1615,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>抑制观测噪声, 输出平滑状态</t>
+          <t>该估计器对传感器送来的观测进行平滑处理，以抑制观测中夹杂的噪声，从而输出平滑、稳定的状态估计值，供后续模块使用。</t>
         </is>
       </c>
       <c r="H24" t="n">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>A/K/B 参数现场标定生效</t>
+          <t>自适应状态估计器允许在机器人现场直接标定A、K、B等模型参数,标定完成之后这些新参数立即生效,并被用于后续的状态估计计算之中。</t>
         </is>
       </c>
       <c r="H25" t="n">
@@ -1713,7 +1713,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>估计残差反馈到校正层 (闭环输入)</t>
+          <t>自适应状态估计器会把估计值与观测值之间的残差反馈给校正层，该残差作为闭环控制的输入，用于修正后续的状态估计。</t>
         </is>
       </c>
       <c r="H26" t="n">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>观测前先猜: x̂₋ = A·x + B·u</t>
+          <t>先验动力学预测器在获得新观测之前先做猜测, 按状态转移方程 x̂₋ = A·x + B·u 推算: 用状态转移矩阵 A 乘当前状态 x, 再加上控制矩阵 B 与控制输入 u 的乘积, 得到下一步的先验状态估计 x̂₋。</t>
         </is>
       </c>
       <c r="H27" t="n">
@@ -1811,7 +1811,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>潜空间恒速速度场 (A=1.0 物理自洽)</t>
+          <t>先验动力学预测器在潜空间里用一个速度恒定不变的速度场来外推未来状态, 该速度场的转移系数 A 取值为 1.0, 使预测满足匀速推进的物理自洽约束, 不会偏离真实运动趋势太远。</t>
         </is>
       </c>
       <c r="H28" t="n">
@@ -1860,7 +1860,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>预测输出作残差基准 (z − x̂₋)</t>
+          <t>该预测器给出预测输出，并把预测输出当作残差的计算基准，用预测输出 z 减去先验状态估计 x̂₋ 得到的差值作为残差信号。</t>
         </is>
       </c>
       <c r="H29" t="n">
@@ -1909,7 +1909,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>A/B 系数标定生效 (物理自洽 A=1.0)</t>
+          <t>先验动力学预测器的A和B两个系数支持现场标定后生效,其中A系数被固定为数值1.0,从而保证动力学预测模型在物理上保持自洽。</t>
         </is>
       </c>
       <c r="H30" t="n">
@@ -1958,7 +1958,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>预测计算零阻塞 (纯 numpy 微秒级)</t>
+          <t>先验动力学预测器的预测计算完全依靠 NumPy 库完成，单次预测的耗时处于微秒量级，因而不会阻塞整体运行流程。</t>
         </is>
       </c>
       <c r="H31" t="n">
@@ -2007,7 +2007,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>r = z − x̂₋ 新息计算</t>
+          <t>状态校正器拿到传感器实测值 z 之后, 计算实测值与先验估计 x̂₋ 之间的差值, 得到新息 r = z − x̂₋, 用这一残差刻画预测与真实的偏离程度, 并驱动后续的状态更新与修正。</t>
         </is>
       </c>
       <c r="H32" t="n">
@@ -2056,7 +2056,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>校正 x̂₊ = x̂₋ + K·r</t>
+          <t>状态校正器把卡尔曼增益 K 乘以新息残差 r 所得的修正量, 叠加到预测阶段得到的先验状态估计值 x̂₋ 上, 得到校正之后的后验估计值 x̂₊, 完成对状态的融合更新。</t>
         </is>
       </c>
       <c r="H33" t="n">
@@ -2105,7 +2105,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>σ(残差·gain) → 接触概率</t>
+          <t>该模块把残差乘以增益得到的结果送入 σ 函数进行变换，σ 函数输出的数值就作为接触发生概率的估计值。</t>
         </is>
       </c>
       <c r="H34" t="n">
@@ -2154,7 +2154,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>残差超阈值 → 异常信号</t>
+          <t>状态校正器把观测值与预测值之间的残差和设定好的阈值进行比较,一旦残差超过阈值,模块就立刻发出异常信号,提醒系统状态出现了偏差。</t>
         </is>
       </c>
       <c r="H35" t="n">
@@ -2203,7 +2203,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>校正后状态喂回预测器 (闭环)</t>
+          <t>状态校正器会把校正之后得到的状态估计值回写给先验动力学预测器，供其作为下一次预测的输入，从而构成闭环。</t>
         </is>
       </c>
       <c r="H36" t="n">
@@ -2252,7 +2252,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>接近→对位→下降→抓取→抬起→转移→插入→完成</t>
+          <t>动作调制器把整条光模块插拔作业拆成八个阶段并依次推进: 接近目标、位置对位、夹爪下降、抓取光模块、抬起、转移至目标位置、对准插入、完成收尾, 前一阶段达成之后才进入下一阶段。</t>
         </is>
       </c>
       <c r="H37" t="n">
@@ -2301,7 +2301,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>前馈+反馈加权合成 u (带否决权)</t>
+          <t>动作调制器把前馈控制器给出的动作分量与反馈控制器给出的动作分量按各自权重加权求和, 合成最终的控制量 u, 同时保留对各分量的否决权, 一旦发现危险动作就将其剔除。</t>
         </is>
       </c>
       <c r="H38" t="n">
@@ -2350,7 +2350,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>各阶段速度上限 V_CAP / 下限 V_MIN</t>
+          <t>该调制器为整个流程的每个运行阶段分别设定速度上限 V_CAP 与速度下限 V_MIN，把各个阶段的执行速度都限制在规定的范围之内。</t>
         </is>
       </c>
       <c r="H39" t="n">
@@ -2399,7 +2399,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>夹持丢失/滑脱 → 自动回退重抓</t>
+          <t>动作调制器持续监测夹爪的夹持状态,一旦发现所夹物体丢失或者从夹爪中滑脱,就自动让机器人回退到原来的安全位置,并重新执行抓取动作。</t>
         </is>
       </c>
       <c r="H40" t="n">
@@ -2448,7 +2448,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>每步决策有依据 (阶段/证据/否决原因)</t>
+          <t>动作调制器在每一步做出的决策都附有明确的依据，这些依据包括当前所处的作业阶段、支持决策的证据以及否决某项动作的原因。</t>
         </is>
       </c>
       <c r="H41" t="n">
@@ -2497,7 +2497,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>saturate ±0.6 物理层限幅</t>
+          <t>安全边界层在动作送出之前对其执行饱和限幅, 把动作向量每个维度的数值都限制在正负 0.6 的物理允许范围以内, 从源头杜绝超出安全边界的指令进入执行环节。</t>
         </is>
       </c>
       <c r="H42" t="n">
@@ -2546,7 +2546,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>速度指令安全上限钳制</t>
+          <t>安全边界层对所有即将下发的速度指令进行上限检查, 一旦指令数值超过预先设定的安全速度上限, 就把它强制钳制在上限值, 确保机械臂的运动速度始终处于安全范围之内。</t>
         </is>
       </c>
       <c r="H43" t="n">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>否决(决策层)+限幅(物理层)+Sys0(硬件) 三层</t>
+          <t>安全执行边界由三层机制联动构成：决策层直接否决危险指令，物理层对输出信号做限幅处理，硬件层的 Sys0 提供最终保护。</t>
         </is>
       </c>
       <c r="H44" t="n">
@@ -2644,7 +2644,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>未夹持末端不穿透台面</t>
+          <t>安全执行边界模块规定,当机械臂末端没有夹持任何物体的时候,末端不允许向下穿透工作台面,从而防止空载的末端撞坏台面或者损坏自身。</t>
         </is>
       </c>
       <c r="H45" t="n">
@@ -2693,7 +2693,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>限幅值/速度上限可标定可追溯</t>
+          <t>安全执行边界的动作限幅值和速度上限等安全参数都可以被标定，并且这些参数的设定数值与修改历史都可以被追溯审计。</t>
         </is>
       </c>
       <c r="H46" t="n">
@@ -2742,7 +2742,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>u_vec 速度指令下发执行层</t>
+          <t>机器人执行器把经过限幅后的动作向量 u_vec 当作速度指令, 正式下发给底层执行层, 由底层执行层据此驱动机械臂与夹爪产生对应的运动。</t>
         </is>
       </c>
       <c r="H47" t="n">
@@ -2791,7 +2791,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>夹爪闭合/张开指令 (gripper_cmd)</t>
+          <t>机器人执行器接收名为 gripper_cmd 的夹爪控制指令, 依据指令中的开合要求驱动夹爪执行闭合或张开动作, 从而在作业流程的适当时机抓住或释放目标工件。</t>
         </is>
       </c>
       <c r="H48" t="n">
@@ -2840,7 +2840,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>执行后状态回读 (位置/夹爪/力)</t>
+          <t>执行器每完成一次动作，该模块就回读执行之后的状态，其中包括末端位置、夹爪状态与受力情况，并把它们作为执行反馈。</t>
         </is>
       </c>
       <c r="H49" t="n">
@@ -2889,7 +2889,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>速度指令 ↔ act ±1 标定 (K_ACT)</t>
+          <t>机器人执行器利用K_ACT这个比例标定系数,在上位机下发的速度指令与取值范围在正负一之间的动作量之间进行相互换算,保证指令与动作准确对应。</t>
         </is>
       </c>
       <c r="H50" t="n">
@@ -2938,7 +2938,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>执行层防抖/防指令风暴</t>
+          <t>机器人执行器会在执行层面加入防抖处理，用来抑制执行动作中的抖动，同时防止高频重复指令不断涌入而形成指令风暴。</t>
         </is>
       </c>
       <c r="H51" t="n">
@@ -2987,7 +2987,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>metaworld env.step 真实 MuJoCo 动力学</t>
+          <t>物理世界模块把机器人执行器送来的动作交给仿真环境, 通过 metaworld 的 env.step 单步接口推进仿真, 由 MuJoCo 引擎按真实物理动力学结算机械臂、夹爪与光模块的位姿变化, 使动作在物理世界中真实生效。</t>
         </is>
       </c>
       <c r="H52" t="n">
@@ -3036,7 +3036,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>夹持/接触力合成 (无力传感器时的几何合成)</t>
+          <t>物理世界模块在没有力传感器的条件下, 依据机械臂与工件之间的几何接触关系来合成夹持力与接触力, 并把推算出的力信息作为反馈数据提供给上层控制环节使用。</t>
         </is>
       </c>
       <c r="H53" t="n">
@@ -3085,7 +3085,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>销/孔/末端位姿物理演化</t>
+          <t>该模块在物理世界中按照力学规律推进销、孔与机械臂末端位姿的演化，让每一步动作都体现为这些对象位置与姿态的实际变化。</t>
         </is>
       </c>
       <c r="H54" t="n">
@@ -3134,7 +3134,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>末端 hand 位置编码器读值 (真机同构)</t>
+          <t>物理世界模块读取机械臂末端手爪上位置编码器的数值,并且按照与真实机器人完全相同的读取方式来读取,保证仿真环境与真机数据同构一致。</t>
         </is>
       </c>
       <c r="H55" t="n">
@@ -3183,7 +3183,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>物理常量/约束与设计一致</t>
+          <t>物理世界模块中使用的物理常量与物理约束都同设计规格保持一致，并且这些常量与约束都可以被审计核对。</t>
         </is>
       </c>
       <c r="H56" t="n">
@@ -3232,7 +3232,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>🎯 能否插入: done + 插入段&lt;0.5s + 末横向错位&lt;0.5mm (12 扰动集; 波形见 📊仿真波形 插深剩余/横向错位格 + 底部验收摘要)</t>
+          <t>物理世界在插入作业结束后判定能否成功: done 完成标志须为真, 插入阶段耗时须小于 0.5 秒, 最终横向错位须小于 0.5 毫米, 三项须在 12 组扰动集上全部成立; 插深剩余量与横向错位的波形见仿真波形面板对应数据格及底部验收摘要。</t>
         </is>
       </c>
       <c r="H57" t="n">
@@ -3281,7 +3281,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>hand/光模块/hole 三类目标检出</t>
+          <t>视觉系统中的目标检测器对每一帧图像执行检测, 从画面中找出机械手、光模块与插孔这三类目标, 输出每个目标的类别标签与在图像中的位置, 供后续解算环节读取。</t>
         </is>
       </c>
       <c r="H58" t="n">
@@ -3330,7 +3330,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>真实 conf 输出 (无写死 0.99)</t>
+          <t>该检测模块对外输出目标检测模型真实计算出的置信度，不再像旧做法那样把置信度直接写死为固定的 0.99。</t>
         </is>
       </c>
       <c r="H59" t="n">
@@ -3379,7 +3379,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>YOLO 权重首次加载缓存 (防播放卡顿)</t>
+          <t>YOLO目标检测模型第一次加载权重时就把权重缓存到内存中,之后每一帧检测都直接使用缓存好的模型,从而避免画面播放过程中出现卡顿现象。</t>
         </is>
       </c>
       <c r="H60" t="n">
@@ -3428,7 +3428,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>遮挡/漏检时诚实标注, 不伪造检测</t>
+          <t>YOLO 目标检测模块在目标物体被遮挡或发生漏检的时候，会如实地标注出当前检测不到目标的状态，而不会伪造虚假的检测结果。</t>
         </is>
       </c>
       <c r="H61" t="n">
@@ -3477,7 +3477,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>单帧 detect_3d 耗时在真实化节奏内</t>
+          <t>视觉系统每收到一帧图像就执行一次 detect_3d 三维目标检测, 单帧处理的总耗时须控制在真实化运行节奏规定的时限以内, 以保证感知的实时性, 不拖慢后续的控制与执行。</t>
         </is>
       </c>
       <c r="H62" t="n">
@@ -3526,7 +3526,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>2D 检测框 → 3D 世界坐标 (深度反投影)</t>
+          <t>视觉系统把图像平面上目标检测框给出的目标位置, 结合深度信息进行反投影解算, 换算成三维空间中的世界坐标, 使机械臂能够依据真实空间位置规划抓取与插入动作。</t>
         </is>
       </c>
       <c r="H63" t="n">
@@ -3575,7 +3575,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>深度模型预测 → 框内中位数深度</t>
+          <t>该模块先让深度模型预测出整幅深度图，再统计目标检测框内各像素的深度值，并取其中位数作为该目标的深度估计结果。</t>
         </is>
       </c>
       <c r="H64" t="n">
@@ -3624,7 +3624,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>cam_mat/fovy/外参精确对齐</t>
+          <t>相机标定把相机内参矩阵、垂直视场角和相机外参这些参数精确标定并相互对齐,保证图像平面上的像素点能够投影到三维空间中的正确位置上。</t>
         </is>
       </c>
       <c r="H65" t="n">
@@ -3673,7 +3673,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>反投影坐标 vs 真值误差量化</t>
+          <t>图像平面到三维空间的解算模块会把图像平面反投影得到的三维坐标与真值坐标进行对比，以此量化解算误差的大小。</t>
         </is>
       </c>
       <c r="H66" t="n">
@@ -3722,7 +3722,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>真机/仿真同一解算链路 (不双轨)</t>
+          <t>视觉系统在真机与仿真环境中共用同一条从图像平面到三维空间的解算链路, 不分别维护两套并行的处理逻辑, 以保证两种场景下二维到三维解算的行为一致、结果可比。</t>
         </is>
       </c>
       <c r="H67" t="n">
@@ -3771,7 +3771,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>夹紧度 1−obs 夹持感知</t>
+          <t>触觉感知模块以夹爪开合状态的观测值为基础, 用一减去该观测值得到夹紧度, 夹紧度数值越大代表夹持越紧, 从而判断工件是否已被夹爪可靠地抓住。</t>
         </is>
       </c>
       <c r="H68" t="n">
@@ -3820,7 +3820,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>接触建立检测 (几何+夹持)</t>
+          <t>该模块根据几何位置关系与夹持状态这两路信号判断接触是否建立，只有当信号满足接触条件时才判定末端已经与工件接触。</t>
         </is>
       </c>
       <c r="H69" t="n">
@@ -3869,7 +3869,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>4D 触觉向量 (grasp/contact 0-1)</t>
+          <t>触觉感知模块把抓取状态和接触状态的信息合成为一个四维触觉向量,向量里每个分量的取值都在零到一之间,用来表示抓持和接触的程度。</t>
         </is>
       </c>
       <c r="H70" t="n">
@@ -3918,7 +3918,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>力觉 → 接触概率语义</t>
+          <t>触觉感知模块会把传感器输出的力觉信号映射为接触概率这一语义，用接触概率的大小来描述当前是否发生了接触。</t>
         </is>
       </c>
       <c r="H71" t="n">
@@ -3967,7 +3967,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>夹持质量 (随动验证) 估计</t>
+          <t>触觉感知系统根据夹爪夹持光模块过程中的触觉反馈估计当前的抓握质量, 并随夹持动作同步进行跟随式验证, 用于判断夹持是否可靠、能否安全进入后续的转移与插入环节。</t>
         </is>
       </c>
       <c r="H72" t="n">
@@ -4016,7 +4016,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>AOI 图像真实处理检出缺陷项</t>
+          <t>外观质量检测模块对拍摄到的 AOI 图像执行真实的图像处理与分析, 从画面中检出存在的各类外观缺陷项, 并输出缺陷判定结论, 供质量记录与拦截处理使用。</t>
         </is>
       </c>
       <c r="H73" t="n">
@@ -4065,7 +4065,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>pass/fail 判定输出</t>
+          <t>该模块根据外观质量检测得到的数据进行最终判定，并对外输出合格或不合格的判定结果，供质量统计参考。</t>
         </is>
       </c>
       <c r="H74" t="n">
@@ -4114,7 +4114,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>打光/曝光/预处理管线</t>
+          <t>外观质量检测模块先控制光源完成打光,再设置好曝光参数拍摄图像,最后经过一套图像预处理流程,把图像整理成便于后续检测的干净画面。</t>
         </is>
       </c>
       <c r="H75" t="n">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>items/缺陷计数汇总</t>
+          <t>外观质量检测模块会汇总本次检测涉及的项目数量与各类缺陷的计数，并输出缺陷项统计结果，供后续的质量判断使用。</t>
         </is>
       </c>
       <c r="H76" t="n">
@@ -4212,7 +4212,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>判定阈值/标准可配置</t>
+          <t>外观质量检测系统把判定光模块外观是否合格的阈值与标准做成可配置项, 使现场人员无需修改程序, 即可按不同批次或客户要求调整外观判定的严苛程度。</t>
         </is>
       </c>
       <c r="H77" t="n">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>MES/自然语言指令 → 任务意图</t>
+          <t>任务规划器接收来自 MES 制造执行系统的指令或操作者给出的自然语言指令, 对指令内容进行语义解析, 提炼出明确的作业任务意图, 作为后续动作规划的总目标。</t>
         </is>
       </c>
       <c r="H78" t="n">
@@ -4310,7 +4310,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>任务意图 → 技能 Token 序列</t>
+          <t>该规划器接收任务意图的描述，把意图转换为由技能 Token 依次排列而成的技能序列，作为后续技能执行的依据。</t>
         </is>
       </c>
       <c r="H79" t="n">
@@ -4359,7 +4359,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Token 必须在库 + 阶段顺序合法</t>
+          <t>任务规划器在生成序列之后会做合法性校验,检查序列里的每个令牌是否都收录在词库中,同时检查各个阶段的先后顺序是否合法,不合格的序列会被拒绝执行。</t>
         </is>
       </c>
       <c r="H80" t="n">
@@ -4408,7 +4408,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>识别作业场景 (五大场景)</t>
+          <t>任务规划器能够从五大作业场景中识别出当前所处的场景，并且把识别得到的结果用于后续的任务规划。</t>
         </is>
       </c>
       <c r="H81" t="n">
@@ -4457,7 +4457,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>规划过程与依据可见</t>
+          <t>任务规划器把规划的生成过程、所依据的条件与最终选择的结果清晰地呈现出来, 让操作人员能够查看每一步任务安排由哪些理由得出, 从而理解并复核机器人的规划结论。</t>
         </is>
       </c>
       <c r="H82" t="n">
@@ -4506,7 +4506,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>力控/对准/插入/未接触分类诊断</t>
+          <t>异常推理器在作业发生异常时, 根据当前的状态与观测特征对异常进行分类诊断, 判断异常属于力控问题、对准问题、插入问题还是未接触问题, 并输出诊断类型供恢复机制参考。</t>
         </is>
       </c>
       <c r="H83" t="n">
@@ -4555,7 +4555,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>每类异常给恢复建议</t>
+          <t>该模块对运行中出现的异常按类型进行归类，并为每一类异常都生成相应的恢复建议，供操作人员或系统参考处理。</t>
         </is>
       </c>
       <c r="H84" t="n">
@@ -4604,7 +4604,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>连续否决/卡死识别</t>
+          <t>异常推理器持续统计某个动作被连续否决的次数,一旦识别出连续否决或者整个流程卡死的情况,就判定系统出现了异常,并触发对应的异常处理。</t>
         </is>
       </c>
       <c r="H85" t="n">
@@ -4653,7 +4653,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>诊断依据 (阶段/残差/接触) 可追溯</t>
+          <t>异常推理器给出的每一条诊断结论都带有可以追溯的诊断依据，这些依据包括当前所处的阶段、状态残差以及接触信息。</t>
         </is>
       </c>
       <c r="H86" t="n">
@@ -4702,7 +4702,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>诊断 → 恢复 → 重试闭环</t>
+          <t>异常推理器在检测到异常之后按诊断、恢复、重试的顺序构成闭环: 先定位异常原因, 再执行恢复动作消除异常, 最后重新尝试受影响的作业环节, 使作业能够自动回到正常流程。</t>
         </is>
       </c>
       <c r="H87" t="n">
@@ -4751,7 +4751,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>场景 → 技能序列 (8 场景)</t>
+          <t>技能编排器根据系统当前所处的作业场景, 在预设的八种场景模板中匹配最合适的技能序列, 再把匹配到的各项技能按顺序编排执行, 以完成当前场景对应的整套作业。</t>
         </is>
       </c>
       <c r="H88" t="n">
@@ -4800,7 +4800,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>performance 参数覆盖默认 (力限/节拍)</t>
+          <t>该编排器在技能执行过程中读取工艺要求的性能参数，用这些参数覆盖系统默认设定，例如力的上限与节拍时间等。</t>
         </is>
       </c>
       <c r="H89" t="n">
@@ -4849,7 +4849,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>原子技能库检索 (242 条/9 类)</t>
+          <t>技能编排器会到原子技能库中进行检索,技能库共收录242条原子技能,这些技能被划分为9个类别,模块从中挑选出适合当前任务的那一条来执行。</t>
         </is>
       </c>
       <c r="H90" t="n">
@@ -4898,7 +4898,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>编排序列合法性校验</t>
+          <t>技能编排器会对编排产生的技能执行序列进行合法性校验，只有校验通过的序列才会被交给后续环节去执行。</t>
         </is>
       </c>
       <c r="H91" t="n">
@@ -4947,7 +4947,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>原子技能可组合成完整作业 (纤维截面)</t>
+          <t>技能编排器把抓取、转移、插入等原子技能当作可独立使用的基础模块, 按当前作业的需要把多个原子技能组合编排成一条完整的光模块插拔作业流程, 实现复杂任务的模块化拼装。</t>
         </is>
       </c>
       <c r="H92" t="n">
@@ -4996,7 +4996,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Kp/阶段速度上限 (引力=快速动作)</t>
+          <t>标定层针对需要快速动作的引力型操作, 标定与之匹配的比例控制增益以及各个作业阶段的速度上限, 使机械臂在执行快速发力动作时既跟得上节奏又不会突破安全速度边界。</t>
         </is>
       </c>
       <c r="H93" t="n">
@@ -5045,7 +5045,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>K_kalman/接触增益/否决阈值 (斥力=状态预测)</t>
+          <t>该标定层负责标定卡尔曼增益 K_kalman、接触增益与否决阈值等参数，并明确此处的斥力数值直接取状态预测的结果。</t>
         </is>
       </c>
       <c r="H94" t="n">
@@ -5094,7 +5094,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>latent_dim/力通道/prior_A 标定</t>
+          <t>标定层对潜空间相关的参数进行标定,这些参数包括潜空间的维度latent_dim、力通道的配置以及先验矩阵prior_A,标定完成之后这些参数即投入后续计算。</t>
         </is>
       </c>
       <c r="H95" t="n">
@@ -5143,7 +5143,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>引力势−斥力势 平衡偏差</t>
+          <t>标定层会计算引力势能与斥力势能之间的差值，并把这一差值作为平衡势的偏差量，用来评估当前的平衡状态。</t>
         </is>
       </c>
       <c r="H96" t="n">
@@ -5192,7 +5192,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>apply_to_engine 精确写回源码字面量</t>
+          <t>标定层通过 apply_to_engine 接口把标定得到的参数精确写回引擎源码, 且写入内容与源码中的字面量写法保持一致, 从而确保新的标定值在引擎中真实生效。</t>
         </is>
       </c>
       <c r="H97" t="n">
@@ -5241,7 +5241,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>误差分解为切向/法向通道</t>
+          <t>接触流形模块把当前的对准误差分解到切向与法向两个通道上, 切向通道负责平行于接触面的偏差, 法向通道负责垂直于接触面的偏差, 分别输出误差分量以指导接触调整。</t>
         </is>
       </c>
       <c r="H98" t="n">
@@ -5290,7 +5290,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>e⊥ 法向偏离风险测量</t>
+          <t>该模块测量接触点在法线方向上的偏离量 e⊥，并以该偏离量的大小作为法向偏离风险的度量依据。</t>
         </is>
       </c>
       <c r="H99" t="n">
@@ -5339,7 +5339,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>e∥ 沿工艺轴进度</t>
+          <t>接触流形模块利用接触点处的切向分量e∥来衡量动作沿工艺轴方向推进的距离,并用这个分量实时追踪当前工序沿工艺轴的完成进度。</t>
         </is>
       </c>
       <c r="H100" t="n">
@@ -5388,7 +5388,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>V=½‖e‖² 李雅普诺夫代价</t>
+          <t>接触流形模块会使用李雅普诺夫代价函数来评估流形代价，该代价函数 V 等于二分之一乘以误差向量的范数平方。</t>
         </is>
       </c>
       <c r="H101" t="n">
@@ -5437,7 +5437,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>接触流形 channel 逐帧发布</t>
+          <t>接触流形模块把每一帧计算得到的接触流形数据封装成消息, 通过专用 channel 逐帧发布出去, 让订阅该 channel 的下游模块能够持续获得最新的接触状态信息。</t>
         </is>
       </c>
       <c r="H102" t="n">
@@ -5486,7 +5486,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>光模块头−孔底 加权二次代价</t>
+          <t>性能流形模块评估机械臂末端夹持的光模块头部与插孔底部之间的对准程度, 用偏差的加权二次代价函数量化失准大小, 代价数值越小表示当前的对准状态越理想。</t>
         </is>
       </c>
       <c r="H103" t="n">
@@ -5535,7 +5535,7 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>高斯光束近似 η=exp(−V/σ²)</t>
+          <t>该模块将耦合过程近似为高斯光束的传播过程，并依据该近似用公式 η=exp(−V/σ²) 计算当前状态所对应的耦合效率 η。</t>
         </is>
       </c>
       <c r="H104" t="n">
@@ -5584,7 +5584,7 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>插入完成态 η 高判据</t>
+          <t>性能流形模块用完成度指标η来判定任务是否完成,当η的数值超过设定的高判据时,系统就认定装配插入动作已经圆满完成。</t>
         </is>
       </c>
       <c r="H105" t="n">
@@ -5633,7 +5633,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>η 低/不升 = 质量退化信号</t>
+          <t>性能流形模块会持续监测性能指标 η，一旦发现 η 的数值偏低或者长期不再上升，就把它视为质量发生退化的信号。</t>
         </is>
       </c>
       <c r="H106" t="n">
@@ -5682,7 +5682,7 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>性能流形地图展示</t>
+          <t>性能流形模块把采集到的各项性能指标组织成流形地图并可视化展示, 使操作人员能够直观查看不同状态下系统性能的分布与走势, 从而把握整体的运行表现。</t>
         </is>
       </c>
       <c r="H107" t="n">
@@ -5731,7 +5731,7 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>引擎轨迹 → 潜状态坐标</t>
+          <t>潜空间模块把仿真引擎输出的原始运动轨迹编码转换为低维的潜状态坐标, 使连续轨迹在潜空间中呈现为紧凑而平滑的状态序列, 供状态预测与技能复用环节直接读取。</t>
         </is>
       </c>
       <c r="H108" t="n">
@@ -5780,7 +5780,7 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>PCA 实测有效维 vs latent_dim</t>
+          <t>该模块对潜空间特征做主成分分析，测出数据实际的有效维数，并与预设的潜空间维度 latent_dim 做对比，检查二者是否一致。</t>
         </is>
       </c>
       <c r="H109" t="n">
@@ -5829,7 +5829,7 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>潜空间速度场 (prior−x̂₋)</t>
+          <t>潜空间模块把先验分布prior与预测得到的先验状态估计x̂₋相减,用两者之间的差值来估计潜空间中的速度场,并据此推进状态的后续演化。</t>
         </is>
       </c>
       <c r="H110" t="n">
@@ -5878,7 +5878,7 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>标定潜维 vs 引擎实际</t>
+          <t>潜空间模块会把标定得到的潜空间维度与实际引擎运行时使用的潜空间维度相互核对，以确保二者保持一致。</t>
         </is>
       </c>
       <c r="H111" t="n">
@@ -5927,7 +5927,7 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>潜状态 channel 逐帧发布</t>
+          <t>潜空间模块把状态估计器维护的潜状态按帧封装成数据消息, 经专用 channel 逐帧发布给下游消费方, 使它们能够实时读取并使用最新的潜状态表示。</t>
         </is>
       </c>
       <c r="H112" t="n">
@@ -28139,7 +28139,7 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>单次前向 111.9µs &lt; 1ms</t>
+          <t>单次前向 107.7µs &lt; 1ms</t>
         </is>
       </c>
     </row>
@@ -32567,7 +32567,7 @@
       </c>
       <c r="E332" t="inlineStr">
         <is>
-          <t>aligned hand=[      0.014       0.597       0.161] peg=[      0.168       0.633       0.012] hole=[     -0.237       0.445       0.126] (真实 align)</t>
+          <t>aligned hand=[      0.038       0.582       0.182] peg=[      0.058       0.648       0.015] hole=[     -0.132       0.643       0.158] (真实 align)</t>
         </is>
       </c>
     </row>
@@ -33809,7 +33809,7 @@
       </c>
       <c r="E378" t="inlineStr">
         <is>
-          <t>多类异常可诊断: {'未接触', '插入未到位'}</t>
+          <t>多类异常可诊断: {'插入未到位', '未接触'}</t>
         </is>
       </c>
     </row>

</xml_diff>